<commit_message>
Caught up to model branch data pipeline changes
</commit_message>
<xml_diff>
--- a/training_data_index.xlsx
+++ b/training_data_index.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Aran\predicty\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamer\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BF1F4A-7EAF-4D1C-A786-F1EDEB4F1D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3D6DB0-3E19-41F6-A026-34E9F8DF8DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="96">
   <si>
     <t>expt</t>
   </si>
@@ -321,12 +321,6 @@
   </si>
   <si>
     <t>distributed_cells</t>
-  </si>
-  <si>
-    <t>mixin60</t>
-  </si>
-  <si>
-    <t>BOGUS</t>
   </si>
 </sst>
 </file>
@@ -724,7 +718,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:T29"/>
+  <dimension ref="A1:T28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.54296875" style="10" bestFit="1" customWidth="1"/>
@@ -1896,13 +1890,13 @@
     </row>
     <row r="22" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="B22" s="7">
-        <v>45354</v>
+        <v>45358</v>
       </c>
       <c r="C22" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="D22" t="s">
         <v>47</v>
@@ -1917,17 +1911,17 @@
         <v>25</v>
       </c>
       <c r="H22" s="8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I22" s="8">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="J22" s="8">
         <v>10</v>
       </c>
       <c r="M22" s="8"/>
       <c r="N22" t="s">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="O22" t="s">
         <v>27</v>
@@ -1945,18 +1939,18 @@
         <v>29</v>
       </c>
       <c r="T22" s="8">
-        <v>229</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B23" s="7">
-        <v>45358</v>
+        <v>45359</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="D23" t="s">
         <v>47</v>
@@ -1965,23 +1959,23 @@
         <v>48</v>
       </c>
       <c r="F23" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="G23" t="s">
         <v>25</v>
       </c>
       <c r="H23" s="8">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I23" s="8">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="J23" s="8">
         <v>10</v>
       </c>
       <c r="M23" s="8"/>
       <c r="N23" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="O23" t="s">
         <v>27</v>
@@ -1999,43 +1993,43 @@
         <v>29</v>
       </c>
       <c r="T23" s="8">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B24" s="7">
-        <v>45359</v>
+        <v>45372</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="D24" t="s">
         <v>47</v>
       </c>
       <c r="E24" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="F24" t="s">
         <v>55</v>
       </c>
       <c r="G24" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="H24" s="8">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="I24" s="8">
-        <v>67</v>
-      </c>
-      <c r="J24" s="8">
-        <v>10</v>
+        <v>24</v>
+      </c>
+      <c r="J24" s="9">
+        <v>1.25</v>
       </c>
       <c r="M24" s="8"/>
       <c r="N24" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="O24" t="s">
         <v>27</v>
@@ -2044,27 +2038,27 @@
         <v>28</v>
       </c>
       <c r="Q24" s="8">
-        <v>420</v>
-      </c>
-      <c r="R24" s="8">
-        <v>2</v>
+        <v>250</v>
+      </c>
+      <c r="R24" s="9">
+        <v>0.75</v>
       </c>
       <c r="S24" t="s">
         <v>29</v>
       </c>
       <c r="T24" s="8">
-        <v>102</v>
+        <v>229</v>
       </c>
     </row>
     <row r="25" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B25" s="7">
-        <v>45372</v>
+        <v>45385</v>
       </c>
       <c r="C25" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="D25" t="s">
         <v>47</v>
@@ -2073,49 +2067,56 @@
         <v>84</v>
       </c>
       <c r="F25" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="G25" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="H25" s="8">
-        <v>75</v>
-      </c>
-      <c r="I25" s="8">
-        <v>24</v>
-      </c>
-      <c r="J25" s="9">
-        <v>1.25</v>
+        <f>4*60+17</f>
+        <v>257</v>
+      </c>
+      <c r="I25" s="9">
+        <v>21.5</v>
+      </c>
+      <c r="J25" s="8">
+        <v>1</v>
+      </c>
+      <c r="K25" t="s">
+        <v>87</v>
+      </c>
+      <c r="L25" t="s">
+        <v>51</v>
       </c>
       <c r="M25" s="8"/>
       <c r="N25" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="O25" t="s">
         <v>27</v>
       </c>
       <c r="P25" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="Q25" s="8">
-        <v>250</v>
+        <v>350</v>
       </c>
       <c r="R25" s="9">
-        <v>0.75</v>
+        <v>1.85</v>
       </c>
       <c r="S25" t="s">
         <v>29</v>
       </c>
       <c r="T25" s="8">
-        <v>229</v>
+        <v>108</v>
       </c>
     </row>
     <row r="26" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B26" s="7">
-        <v>45385</v>
+        <v>45397</v>
       </c>
       <c r="C26" t="s">
         <v>21</v>
@@ -2124,51 +2125,44 @@
         <v>47</v>
       </c>
       <c r="E26" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="F26" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="G26" t="s">
         <v>25</v>
       </c>
       <c r="H26" s="8">
-        <f>4*60+17</f>
-        <v>257</v>
-      </c>
-      <c r="I26" s="9">
-        <v>21.5</v>
+        <v>12</v>
+      </c>
+      <c r="I26" s="8">
+        <v>24</v>
       </c>
       <c r="J26" s="8">
-        <v>1</v>
-      </c>
-      <c r="K26" t="s">
-        <v>87</v>
-      </c>
-      <c r="L26" t="s">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="M26" s="8"/>
       <c r="N26" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="O26" t="s">
         <v>27</v>
       </c>
       <c r="P26" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="Q26" s="8">
         <v>350</v>
       </c>
-      <c r="R26" s="9">
-        <v>1.85</v>
+      <c r="R26" s="8">
+        <v>2</v>
       </c>
       <c r="S26" t="s">
         <v>29</v>
       </c>
       <c r="T26" s="8">
-        <v>108</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -2179,7 +2173,7 @@
         <v>45397</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="D27" t="s">
         <v>47</v>
@@ -2194,17 +2188,21 @@
         <v>25</v>
       </c>
       <c r="H27" s="8">
-        <v>12</v>
+        <f>24*60+32</f>
+        <v>1472</v>
       </c>
       <c r="I27" s="8">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J27" s="8">
         <v>10</v>
       </c>
+      <c r="L27" t="s">
+        <v>51</v>
+      </c>
       <c r="M27" s="8"/>
       <c r="N27" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="O27" t="s">
         <v>27</v>
@@ -2222,34 +2220,33 @@
         <v>29</v>
       </c>
       <c r="T27" s="8">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B28" s="7">
-        <v>45397</v>
+        <v>45411</v>
       </c>
       <c r="C28" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="D28" t="s">
         <v>47</v>
       </c>
       <c r="E28" t="s">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="F28" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="G28" t="s">
         <v>25</v>
       </c>
       <c r="H28" s="8">
-        <f>24*60+32</f>
-        <v>1472</v>
+        <v>70</v>
       </c>
       <c r="I28" s="8">
         <v>23</v>
@@ -2257,12 +2254,9 @@
       <c r="J28" s="8">
         <v>10</v>
       </c>
-      <c r="L28" t="s">
-        <v>51</v>
-      </c>
       <c r="M28" s="8"/>
       <c r="N28" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="O28" t="s">
         <v>27</v>
@@ -2271,7 +2265,7 @@
         <v>28</v>
       </c>
       <c r="Q28" s="8">
-        <v>350</v>
+        <v>420</v>
       </c>
       <c r="R28" s="8">
         <v>2</v>
@@ -2280,60 +2274,6 @@
         <v>29</v>
       </c>
       <c r="T28" s="8">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B29" s="7">
-        <v>45411</v>
-      </c>
-      <c r="C29" t="s">
-        <v>73</v>
-      </c>
-      <c r="D29" t="s">
-        <v>47</v>
-      </c>
-      <c r="E29" t="s">
-        <v>94</v>
-      </c>
-      <c r="F29" t="s">
-        <v>39</v>
-      </c>
-      <c r="G29" t="s">
-        <v>25</v>
-      </c>
-      <c r="H29" s="8">
-        <v>70</v>
-      </c>
-      <c r="I29" s="8">
-        <v>23</v>
-      </c>
-      <c r="J29" s="8">
-        <v>10</v>
-      </c>
-      <c r="M29" s="8"/>
-      <c r="N29" t="s">
-        <v>95</v>
-      </c>
-      <c r="O29" t="s">
-        <v>27</v>
-      </c>
-      <c r="P29" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q29" s="8">
-        <v>420</v>
-      </c>
-      <c r="R29" s="8">
-        <v>2</v>
-      </c>
-      <c r="S29" t="s">
-        <v>29</v>
-      </c>
-      <c r="T29" s="8">
         <v>90</v>
       </c>
     </row>

</xml_diff>